<commit_message>
Update the bundled master with the 17 newly filled pictures.
Co-authored-by: ngaadmin <ngaadmin@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/lib/academy/lessons/payload/source/master/module-1-screens.xlsx
+++ b/lib/academy/lessons/payload/source/master/module-1-screens.xlsx
@@ -5885,7 +5885,11 @@
           <t>Holly promised Pippa a $20 board game for her birthday on Saturday. Holly only has the $10 she kept safe. True or false: she can buy it now.</t>
         </is>
       </c>
-      <c r="F14" s="5" t="n"/>
+      <c r="F14" s="5" t="inlineStr">
+        <is>
+          <t>holly-deciding-512.webp</t>
+        </is>
+      </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
           <t>CORRECT: False</t>
@@ -6209,7 +6213,11 @@
           <t>It's Saturday, Pippa's birthday, and the party is about to start. Drag the gift to Pippa so Holly can keep her promise.</t>
         </is>
       </c>
-      <c r="F21" s="5" t="n"/>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>beat-pf-m1-l2-r6-app.webp</t>
+        </is>
+      </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
           <t>SOURCE: concept-gift-box
@@ -6423,7 +6431,11 @@
           <t>She accidentally breaks Pippa's headphones. What's the problem Holly faces?</t>
         </is>
       </c>
-      <c r="F26" s="5" t="n"/>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>beat-pf-m1-l3-r5-app.webp</t>
+        </is>
+      </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
           <t>CHOICE A: 💸 Holly has no money for a new pair.
@@ -7047,7 +7059,11 @@
           <t>After practice, Holly walks home past the stores. Every window seems to be shouting at her.</t>
         </is>
       </c>
-      <c r="F40" s="5" t="n"/>
+      <c r="F40" s="5" t="inlineStr">
+        <is>
+          <t>holly-walking-512.webp</t>
+        </is>
+      </c>
       <c r="G40" s="5" t="n"/>
       <c r="H40" s="5" t="n"/>
       <c r="I40" s="5" t="inlineStr">
@@ -7462,7 +7478,11 @@
           <t>It's Senna's birthday, and the gelato shop has a birthday deal. Senna wants Holly to get one too. For Holly, her own gelato is a ______.</t>
         </is>
       </c>
-      <c r="F49" s="5" t="n"/>
+      <c r="F49" s="5" t="inlineStr">
+        <is>
+          <t>prop-ex-m1-gelato-r3.webp</t>
+        </is>
+      </c>
       <c r="G49" s="5" t="inlineStr">
         <is>
           <t>OPTIONS: 🍦 want | ✅ need | 🧾 bill
@@ -7950,7 +7970,11 @@
           <t>Senna asks Holly to the movies. The ticket and popcorn cost $18, and Mom will pay half. Holly has saved $12 from her allowance. Can she pay her half?</t>
         </is>
       </c>
-      <c r="F60" s="5" t="n"/>
+      <c r="F60" s="5" t="inlineStr">
+        <is>
+          <t>prop-mv-m1-group-movie-day-r2-app.webp</t>
+        </is>
+      </c>
       <c r="G60" s="5" t="inlineStr">
         <is>
           <t>CHOICE A: ✅ Yes, she has enough
@@ -8275,7 +8299,11 @@
           <t>At the ticket counter, Mom pays her half. Drag Holly's $9 to the counter.</t>
         </is>
       </c>
-      <c r="F67" s="5" t="n"/>
+      <c r="F67" s="5" t="inlineStr">
+        <is>
+          <t>prop-mv-m1-group-movie-day-r2-app.webp</t>
+        </is>
+      </c>
       <c r="G67" s="5" t="inlineStr">
         <is>
           <t>SOURCE: 💵 $9
@@ -8485,7 +8513,11 @@
           <t>Holly and Senna walk past a café with a bubble tea deal, on today only. Before reaching for her wallet, Holly ______.</t>
         </is>
       </c>
-      <c r="F72" s="5" t="n"/>
+      <c r="F72" s="5" t="inlineStr">
+        <is>
+          <t>prop-pf-m1-bubble-tea-r1.webp</t>
+        </is>
+      </c>
       <c r="G72" s="5" t="inlineStr">
         <is>
           <t>OPTIONS: 🧠 stops and thinks | 🛍️ buys it straight away | 🙋 asks Senna to pay
@@ -8719,7 +8751,11 @@
           <t>What if the bubble tea cost $7? After her share, Holly has $6. Can she buy her own?</t>
         </is>
       </c>
-      <c r="F77" s="5" t="n"/>
+      <c r="F77" s="5" t="inlineStr">
+        <is>
+          <t>beat-pf-m1-l7-r5-app.webp</t>
+        </is>
+      </c>
       <c r="G77" s="5" t="inlineStr">
         <is>
           <t>CHOICE A: ❌ No, she's $1 short
@@ -9752,7 +9788,11 @@
           <t>The group happily agrees, and Senna makes popcorn. Holly joins in and still has {cash}.</t>
         </is>
       </c>
-      <c r="F100" s="5" t="n"/>
+      <c r="F100" s="5" t="inlineStr">
+        <is>
+          <t>beat-pf-m1-l6-r5-app.webp</t>
+        </is>
+      </c>
       <c r="G100" s="5" t="inlineStr">
         <is>
           <t>CONTINUE → GO Screen 8</t>
@@ -11172,6 +11212,11 @@
           <t>It's Saturday, Max's birthday, and the party is about to start. Drag the gift to Max so Senna can keep his promise.</t>
         </is>
       </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>beat-mv-m1-l2-r6-app.webp</t>
+        </is>
+      </c>
       <c r="G21" s="6" t="inlineStr">
         <is>
           <t>SOURCE: concept-gift-box
@@ -11365,6 +11410,11 @@
       <c r="E26" s="6" t="inlineStr">
         <is>
           <t>He accidentally breaks Max's headphones. What's the problem Senna faces?</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>beat-mv-m1-l3-r5-app.webp</t>
         </is>
       </c>
       <c r="G26" s="6" t="inlineStr">
@@ -12335,6 +12385,11 @@
           <t>It's Saskia's birthday, and the gelato shop has a birthday deal. Saskia wants Senna to get one too. For Senna, his own gelato is a ______.</t>
         </is>
       </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>prop-ex-m1-gelato-r3.webp</t>
+        </is>
+      </c>
       <c r="G49" s="6" t="inlineStr">
         <is>
           <t>OPTIONS: 🍦 want | ✅ need | 🧾 bill
@@ -12784,6 +12839,11 @@
           <t>Saskia asks Senna to the movies. The ticket and popcorn cost $30, and Mom will pay half. Senna has saved $18 of spending money. Can he pay his half?</t>
         </is>
       </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>prop-mv-m1-group-movie-day-r2-app.webp</t>
+        </is>
+      </c>
       <c r="G60" s="6" t="inlineStr">
         <is>
           <t>CHOICE A: ✅ Yes, he has enough
@@ -13091,6 +13151,11 @@
           <t>At the ticket counter, Mom pays her half. Drag Senna's $15 to the counter.</t>
         </is>
       </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>beat-mv-m1-l6-r5-app.webp</t>
+        </is>
+      </c>
       <c r="G67" s="6" t="inlineStr">
         <is>
           <t>SOURCE: 💵 $15
@@ -13279,6 +13344,11 @@
       <c r="E72" s="6" t="inlineStr">
         <is>
           <t>Senna and Saskia walk past a juice bar with a smoothie deal, on today only. Before reaching for his wallet, Senna ______.</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>prop-mv-m1-group-big-news-r1-app.webp</t>
         </is>
       </c>
       <c r="G72" s="6" t="inlineStr">
@@ -13498,6 +13568,11 @@
       <c r="E77" s="6" t="inlineStr">
         <is>
           <t>What if the smoothie cost $9? After his share, Senna has $8. Can he buy his own?</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>beat-mv-m1-l7-r5-app.webp</t>
         </is>
       </c>
       <c r="G77" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Swap in the f6ff7ed9 master and the four new Module 1 pictures.
Pathfinder and Maverick pick up the new pair files, Explorer lesson 1 uses the lemonade family scene, and the binned family intro file is removed. The reader still selects the M1 tabs by name, so Sheet1 is ignored.

Co-authored-by: ngaadmin <ngaadmin@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/lib/academy/lessons/payload/source/master/module-1-screens.xlsx
+++ b/lib/academy/lessons/payload/source/master/module-1-screens.xlsx
@@ -3,25 +3,26 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="29400" yWindow="500" windowWidth="38400" windowHeight="21100" tabRatio="600" firstSheet="0" activeTab="3" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="29400" yWindow="0" windowWidth="38400" windowHeight="21600" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M1 Explorer" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M1 Pathfinder" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M1 Maverick" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M2 Explorer" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M2 Pathfinder" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M2 Maverick" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lesson Details" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M1 Pathfinder" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M1 Maverick" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M2 Explorer" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M2 Pathfinder" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M2 Maverick" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lesson Details" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'M1 Explorer'!$A$1:$K$102</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'M1 Pathfinder'!$A$1:$K$111</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'M1 Maverick'!$A$1:$K$111</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'M2 Explorer'!$A$1:$K$102</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'M2 Pathfinder'!$A$1:$K$102</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'M2 Maverick'!$A$1:$K$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Lesson Details'!$A$1:$J$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'M1 Pathfinder'!$A$1:$K$111</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'M1 Maverick'!$A$1:$K$111</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'M2 Explorer'!$A$1:$K$102</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'M2 Pathfinder'!$A$1:$K$102</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'M2 Maverick'!$A$1:$K$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Lesson Details'!$A$1:$J$28</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -57,7 +58,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -67,12 +68,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFC7CE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -89,7 +84,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -107,9 +102,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -620,7 +612,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>explorer-m1-l1-intro-lars-family-r2.webp</t>
+          <t>lemonade-family-scene-r10.webp</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -5066,6 +5058,422 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A57"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="16" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Explorer Image</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>lemonade-family-scene-r10.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="32" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>explorer-m1-l1-intro-lars-family-r2.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="16" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>lars-senna-chatting.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="16" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>concept-coin-stack.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="16" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>concept-wallet.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="16" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>em1-02-l1r7-senna-coins-r3.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="16" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>concept-piggy-bank.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="16" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>lars-senna-sidebyside.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="32" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>em1-03-l1r11-lars-lemonade-r3.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="16" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>medal-skill1-bronze-app.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="16" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>beat-ex-m1-l2-r1.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="16" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>concept-gift-box.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="32" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>em1-05-l2r21-lars-mom-supplies-r1.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="16" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>prop-ex-m1-wallet-r1.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="16" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>lars-deciding-512.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="32" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>em1-04-l2r20-lars-mom-bike-note-r3.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="16" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>prop-ex-m1-stand-set-r1.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="16" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>medal-skill2-bronze-app.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="16" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>beat-ex-m1-l3-r1.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="32" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>prop-ex-m1-emergencies-jar-r1.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="32" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>em1-06-l3r27-emergencies-jar-r1.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="16" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>lars-mason-chatting-512.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="16" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>medal-skill3-bronze.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="16" customHeight="1">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>beat-ex-m1-l4-r1.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="16" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>lars-mason-sidebyside-512.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="16" customHeight="1">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>lars-mason-chatting.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="32" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>em1-09-l4r41-saving-stand-dream-r1.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="16" customHeight="1">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>fishing-rod-sign.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="16" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>concept-growth-chart.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="32" customHeight="1">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>em1-08-l4r45-startup-envelope-r3.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="16" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>medal-skill1-silver.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="16" customHeight="1">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>beat-ex-m1-l5-r4.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="16" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>lars-mia-sidebyside.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="32" customHeight="1">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>em1-10-l5r50-lars-mia-gelato-r1.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="16" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>lars-thinking-512.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="16" customHeight="1">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>prop-ex-m1-gelato-r3.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="16" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>lars-mia-chatting.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="16" customHeight="1">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>medal-skill2-silver.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="16" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>beat-ex-m1-l6-r1.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="32" customHeight="1">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>em1-11-l6r59-lars-movie-ticket-r1.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="32" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>em1-12-l6r60-mia-lemon-doodle-r1.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="16" customHeight="1">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>prop-ex-m1-lemon-ticket-r4.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="16" customHeight="1">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>medal-skill3-silver.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="16" customHeight="1">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>beat-ex-m1-l7-r1.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="32" customHeight="1">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>em1-15-l7r72-lars-bike-dream-r1.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="32" customHeight="1">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>em1-16-l7r73-lars-wallet-mall-r1.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="16" customHeight="1">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>prop-ex-m1-slushie-r2.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="16" customHeight="1">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>lars-waving-512.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="16" customHeight="1">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>prop-ex-m1-bike-bubble-r1.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="16" customHeight="1">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>beat-ex-m1-l8-r2.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="16" customHeight="1">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>lars-mason-sidebyside.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="32" customHeight="1">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>em1-07-l3r31-lars-mason-empty-wallet-r1.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="32" customHeight="1">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>em1-18-l9r103-lars-closer-to-bike-r1.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="16" customHeight="1">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>beat-ex-m1-l9-r1.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="32" customHeight="1">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>em1-17-l9r102-lemonade-stand-open-r1.webp</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="16" customHeight="1">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>lars-celebrating-512.webp</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5743,7 +6151,7 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>holly-thinking-512.webp</t>
+          <t>prop-pf-m1-startup-kit-r2.webp</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
@@ -6402,7 +6810,7 @@
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>holly-celebrating-512.webp</t>
+          <t>concept-coin-stack.webp</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
@@ -6719,7 +7127,7 @@
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>holly-walking-512.webp</t>
+          <t>prop-pf-m1-startup-kit-r2.webp</t>
         </is>
       </c>
       <c r="G40" s="5" t="n"/>
@@ -7132,7 +7540,7 @@
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>holly-deciding-512.webp</t>
+          <t>holly-senna-chatting-r1-512.webp</t>
         </is>
       </c>
       <c r="G50" s="5" t="inlineStr">
@@ -7577,7 +7985,7 @@
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>holly-thinking-512.webp</t>
+          <t>prop-pf-m1-paw-ticket-r2.webp</t>
         </is>
       </c>
       <c r="G61" s="5" t="inlineStr">
@@ -7710,7 +8118,7 @@
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>holly-hands-on-hips-512.webp</t>
+          <t>holly-senna-chatting-r1-512.webp</t>
         </is>
       </c>
       <c r="G64" s="5" t="inlineStr">
@@ -8059,7 +8467,7 @@
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
-          <t>holly-thinking-512.webp</t>
+          <t>prop-pf-m1-trip-bubble-r1.webp</t>
         </is>
       </c>
       <c r="G73" s="5" t="inlineStr">
@@ -8102,7 +8510,7 @@
       </c>
       <c r="F74" s="5" t="inlineStr">
         <is>
-          <t>holly-hands-on-hips-512.webp</t>
+          <t>prop-ex-m1-wallet-r1.webp</t>
         </is>
       </c>
       <c r="G74" s="5" t="inlineStr">
@@ -8502,7 +8910,7 @@
       </c>
       <c r="F84" s="5" t="inlineStr">
         <is>
-          <t>holly-walking-512.webp</t>
+          <t>prop-ex-m1-wallet-r1.webp</t>
         </is>
       </c>
       <c r="G84" s="5" t="inlineStr">
@@ -8962,7 +9370,7 @@
       </c>
       <c r="F95" s="5" t="inlineStr">
         <is>
-          <t>holly-walking-512.webp</t>
+          <t>concept-wallet.webp</t>
         </is>
       </c>
       <c r="G95" s="5" t="inlineStr">
@@ -9291,7 +9699,7 @@
       </c>
       <c r="F103" s="5" t="inlineStr">
         <is>
-          <t>holly-celebrating-512.webp</t>
+          <t>prop-pf-m1-trip-bubble-r1.webp</t>
         </is>
       </c>
       <c r="G103" s="5" t="inlineStr">
@@ -9507,7 +9915,7 @@
       </c>
       <c r="F108" s="5" t="inlineStr">
         <is>
-          <t>holly-sitting-512.webp</t>
+          <t>prop-pf-m1-beagle-r1.webp</t>
         </is>
       </c>
       <c r="G108" s="5" t="inlineStr">
@@ -9651,7 +10059,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -9671,8 +10079,8 @@
     <col width="50" customWidth="1" style="6" min="9" max="9"/>
     <col width="45" customWidth="1" style="6" min="10" max="10"/>
     <col width="18" customWidth="1" style="6" min="11" max="11"/>
-    <col width="8.83203125" customWidth="1" style="6" min="12" max="14"/>
-    <col width="8.83203125" customWidth="1" style="6" min="15" max="16384"/>
+    <col width="8.83203125" customWidth="1" style="6" min="12" max="15"/>
+    <col width="8.83203125" customWidth="1" style="6" min="16" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -9943,7 +10351,7 @@
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>beat-mv-m1-l1-r6-app.webp</t>
+          <t>prop-mv-m1-group-money-r1-app.webp</t>
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr">
@@ -10098,7 +10506,7 @@
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>senna-older-thinking-r1-512.webp</t>
+          <t>mv-m1-03-l1r11-senna-video-plan-r3.webp</t>
         </is>
       </c>
       <c r="I11" s="6" t="inlineStr">
@@ -10283,7 +10691,7 @@
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>senna-older-thinking-r1-512.webp</t>
+          <t>prop-mv-m1-tripod-r1-app.webp</t>
         </is>
       </c>
       <c r="G16" s="6" t="inlineStr">
@@ -10511,7 +10919,7 @@
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>prop-mv-m1-camera-bubble-r2.webp</t>
+          <t>prop-mv-m1-group-plan-r1-app.webp</t>
         </is>
       </c>
       <c r="I22" s="6" t="inlineStr">
@@ -10875,7 +11283,7 @@
       </c>
       <c r="F32" s="6" t="inlineStr">
         <is>
-          <t>senna-older-celebrating-r1-512.webp</t>
+          <t>prop-mv-m1-group-headphones-r1-app.webp</t>
         </is>
       </c>
       <c r="G32" s="6" t="inlineStr">
@@ -11158,7 +11566,7 @@
       </c>
       <c r="F40" s="6" t="inlineStr">
         <is>
-          <t>senna-older-walking-r1-512.webp</t>
+          <t>prop-mv-m1-group-startup-kit-r2-app.webp</t>
         </is>
       </c>
       <c r="K40" s="6" t="inlineStr">
@@ -11359,7 +11767,7 @@
       </c>
       <c r="F45" s="6" t="inlineStr">
         <is>
-          <t>senna-older-celebrating-r1-512.webp</t>
+          <t>mv-m1-08-l4r45-senna-startup-envelope-r4.webp</t>
         </is>
       </c>
       <c r="K45" s="6" t="inlineStr">
@@ -11527,7 +11935,7 @@
       </c>
       <c r="F50" s="6" t="inlineStr">
         <is>
-          <t>senna-older-deciding-r1-512.webp</t>
+          <t>prop-mv-m1-group-startup-kit-r2-app.webp</t>
         </is>
       </c>
       <c r="G50" s="6" t="inlineStr">
@@ -11927,7 +12335,7 @@
       </c>
       <c r="F61" s="6" t="inlineStr">
         <is>
-          <t>senna-older-thinking-r1-512.webp</t>
+          <t>prop-mv-m1-camera-ticket-r2.webp</t>
         </is>
       </c>
       <c r="G61" s="6" t="inlineStr">
@@ -12048,7 +12456,7 @@
       </c>
       <c r="F64" s="6" t="inlineStr">
         <is>
-          <t>senna-older-hands-on-hips-r1-512.webp</t>
+          <t>prop-mv-m1-group-movie-day-r2-app.webp</t>
         </is>
       </c>
       <c r="G64" s="6" t="inlineStr">
@@ -12353,7 +12761,7 @@
       </c>
       <c r="F73" s="6" t="inlineStr">
         <is>
-          <t>senna-older-thinking-r1-512.webp</t>
+          <t>prop-mv-m1-camera-bubble-r2.webp</t>
         </is>
       </c>
       <c r="G73" s="6" t="inlineStr">
@@ -12392,7 +12800,7 @@
       </c>
       <c r="F74" s="6" t="inlineStr">
         <is>
-          <t>senna-older-hands-on-hips-r1-512.webp</t>
+          <t>prop-mv-m1-group-money-r1-app.webp</t>
         </is>
       </c>
       <c r="G74" s="6" t="inlineStr">
@@ -12746,7 +13154,7 @@
       </c>
       <c r="F84" s="6" t="inlineStr">
         <is>
-          <t>senna-older-walking-r1-512.webp</t>
+          <t>prop-mv-m1-group-money-r1-app.webp</t>
         </is>
       </c>
       <c r="G84" s="6" t="inlineStr">
@@ -13167,7 +13575,7 @@
       </c>
       <c r="F95" s="6" t="inlineStr">
         <is>
-          <t>senna-older-walking-r1-512.webp</t>
+          <t>concept-wallet.webp</t>
         </is>
       </c>
       <c r="G95" s="6" t="inlineStr">
@@ -13463,7 +13871,7 @@
       </c>
       <c r="F103" s="6" t="inlineStr">
         <is>
-          <t>senna-older-celebrating-r1-512.webp</t>
+          <t>prop-mv-m1-camera-bubble-r2.webp</t>
         </is>
       </c>
       <c r="G103" s="6" t="inlineStr">
@@ -13659,7 +14067,7 @@
       </c>
       <c r="F108" s="6" t="inlineStr">
         <is>
-          <t>senna-older-sitting-r1-512.webp</t>
+          <t>prop-mv-m1-tripod-r1-app.webp</t>
         </is>
       </c>
       <c r="G108" s="6" t="inlineStr">
@@ -13786,7 +14194,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -13806,7 +14214,8 @@
     <col width="50" customWidth="1" style="6" min="9" max="9"/>
     <col width="45" customWidth="1" style="6" min="10" max="10"/>
     <col width="18" customWidth="1" style="6" min="11" max="11"/>
-    <col width="8.83203125" customWidth="1" style="6" min="12" max="16384"/>
+    <col width="8.83203125" customWidth="1" style="6" min="12" max="12"/>
+    <col width="8.83203125" customWidth="1" style="6" min="13" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -13877,7 +14286,7 @@
           <t>Scenario Beat</t>
         </is>
       </c>
-      <c r="E2" s="8" t="inlineStr">
+      <c r="E2" s="7" t="inlineStr">
         <is>
           <t>It's Lars's first Saturday as a lemonade seller.
 Mom and Dad told the neighbors, so they know his stand is open. Now he just hopes they'll stop by and buy some.</t>
@@ -14063,7 +14472,6 @@
 CORRECT: A</t>
         </is>
       </c>
-      <c r="I7" s="6" t="n"/>
     </row>
     <row r="8" ht="80" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
@@ -14472,7 +14880,6 @@
           <t>Lars pats the $12 in his pocket and grins. This morning, people walked right past. Then he smiled, spoke up and asked, and six thirsty soccer players said yes!</t>
         </is>
       </c>
-      <c r="I20" s="6" t="n"/>
     </row>
     <row r="21" ht="16" customHeight="1">
       <c r="A21" s="6" t="inlineStr">
@@ -14661,7 +15068,6 @@
           <t>Not quite! Some of his earnings had to buy next week's lemons and cups, so not all of it was savings for his bike goal. Try again!</t>
         </is>
       </c>
-      <c r="I26" s="6" t="n"/>
     </row>
     <row r="27" ht="32" customHeight="1">
       <c r="A27" s="6" t="inlineStr">
@@ -17070,7 +17476,6 @@
 His bike money is growing, one scrap of paper at a time.</t>
         </is>
       </c>
-      <c r="I100" s="6" t="n"/>
     </row>
     <row r="101" ht="64" customHeight="1">
       <c r="A101" s="6" t="inlineStr">
@@ -17133,7 +17538,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -17223,7 +17628,7 @@
           <t>Scenario Beat</t>
         </is>
       </c>
-      <c r="E2" s="8" t="inlineStr">
+      <c r="E2" s="7" t="inlineStr">
         <is>
           <t>It's Holly's first week as a dog walker.
 Mom told the neighbors, and Holly put a flyer in every mailbox on their block. Now she just hopes they'll call and book a walk.</t>
@@ -20475,7 +20880,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -20560,7 +20965,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Swap in the 206ed0cc master so lesson 1 opens on a chat, then a celebrate.
Row 3 is the chatting pair and row 4 is the celebrating pose in every cohort. Maverick rows 11 and 45 use the tripod and group-money pictures, and the two replaced scene files are removed.

Co-authored-by: ngaadmin <ngaadmin@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/lib/academy/lessons/payload/source/master/module-1-screens.xlsx
+++ b/lib/academy/lessons/payload/source/master/module-1-screens.xlsx
@@ -612,7 +612,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>lemonade-family-scene-r10.webp</t>
+          <t>lars-senna-chatting.webp</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -654,7 +654,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>lars-senna-chatting.webp</t>
+          <t>lars-celebrating-512.webp</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -5618,7 +5618,7 @@
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>beat-pf-m1-l1-r8-app.webp</t>
+          <t>holly-senna-chatting-r1-512.webp</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
@@ -5660,7 +5660,7 @@
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>holly-senna-chatting-r1-512.webp</t>
+          <t>holly-celebrating-512.webp</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
@@ -10201,7 +10201,7 @@
       </c>
       <c r="F3" s="6" t="inlineStr">
         <is>
-          <t>beat-mv-m1-l1-r6-app.webp</t>
+          <t>senna-older-max-chatting-r1-512.webp</t>
         </is>
       </c>
       <c r="G3" s="6" t="inlineStr">
@@ -10239,7 +10239,7 @@
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>senna-older-max-chatting-r1-512.webp</t>
+          <t>senna-older-celebrating-r1-512.webp</t>
         </is>
       </c>
       <c r="G4" s="6" t="inlineStr">
@@ -10506,7 +10506,7 @@
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>mv-m1-03-l1r11-senna-video-plan-r3.webp</t>
+          <t>prop-mv-m1-tripod-r1-app.webp</t>
         </is>
       </c>
       <c r="I11" s="6" t="inlineStr">
@@ -11767,7 +11767,7 @@
       </c>
       <c r="F45" s="6" t="inlineStr">
         <is>
-          <t>mv-m1-08-l4r45-senna-startup-envelope-r4.webp</t>
+          <t>prop-mv-m1-group-money-r1-app.webp</t>
         </is>
       </c>
       <c r="K45" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Swap in the f6602939 master and the revised prop stills.
Column F now names the 20 new WebP files. Screens1.csv image columns match that sheet. The two flattened r1 props are removed because nothing still names them.

Co-authored-by: ngaadmin <ngaadmin@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/lib/academy/lessons/payload/source/master/module-1-screens.xlsx
+++ b/lib/academy/lessons/payload/source/master/module-1-screens.xlsx
@@ -3,26 +3,25 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="29400" yWindow="0" windowWidth="38400" windowHeight="21600" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="29400" yWindow="500" windowWidth="38400" windowHeight="20040" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M1 Explorer" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M1 Pathfinder" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M1 Maverick" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M2 Explorer" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M2 Pathfinder" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M2 Maverick" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lesson Details" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M1 Pathfinder" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M1 Maverick" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M2 Explorer" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M2 Pathfinder" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="M2 Maverick" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lesson Details" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'M1 Explorer'!$A$1:$K$102</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'M1 Pathfinder'!$A$1:$K$111</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'M1 Maverick'!$A$1:$K$111</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'M2 Explorer'!$A$1:$K$102</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'M2 Pathfinder'!$A$1:$K$102</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'M2 Maverick'!$A$1:$K$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Lesson Details'!$A$1:$J$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'M1 Pathfinder'!$A$1:$K$111</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'M1 Maverick'!$A$1:$K$111</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'M2 Explorer'!$A$1:$K$102</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'M2 Pathfinder'!$A$1:$K$102</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'M2 Maverick'!$A$1:$K$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Lesson Details'!$A$1:$J$28</definedName>
   </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
@@ -1189,7 +1188,7 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>prop-ex-m1-wallet-r1.webp</t>
+          <t>prop-ex-m1-wallet-r2.webp</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
@@ -1429,7 +1428,7 @@
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>prop-ex-m1-stand-set-r1.webp</t>
+          <t>prop-ex-m1-stand-set-r2.webp</t>
         </is>
       </c>
       <c r="G23" s="2" t="n"/>
@@ -1711,7 +1710,7 @@
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>prop-ex-m1-emergencies-jar-r1.webp</t>
+          <t>prop-ex-m1-emergencies-jar-r2.webp</t>
         </is>
       </c>
       <c r="G30" s="2" t="n"/>
@@ -2372,7 +2371,7 @@
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
-          <t>prop-ex-m1-stand-set-r1.webp</t>
+          <t>prop-ex-m1-stand-set-r2.webp</t>
         </is>
       </c>
       <c r="G46" s="2" t="n"/>
@@ -2618,7 +2617,7 @@
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
-          <t>prop-ex-m1-gelato-r3.webp</t>
+          <t>prop-ex-m1-gelato-r4.webp</t>
         </is>
       </c>
       <c r="G52" s="2" t="inlineStr">
@@ -2697,7 +2696,7 @@
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>prop-ex-m1-wallet-r1.webp</t>
+          <t>prop-ex-m1-wallet-r2.webp</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -3192,7 +3191,7 @@
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>prop-ex-m1-lemon-ticket-r4.webp</t>
+          <t>prop-ex-m1-lemon-ticket-r5.webp</t>
         </is>
       </c>
       <c r="G66" s="2" t="n"/>
@@ -3303,7 +3302,7 @@
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>prop-ex-m1-lemon-ticket-r4.webp</t>
+          <t>prop-ex-m1-lemon-ticket-r5.webp</t>
         </is>
       </c>
       <c r="G69" s="2" t="n"/>
@@ -3787,7 +3786,7 @@
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
-          <t>prop-ex-m1-bike-bubble-r1.webp</t>
+          <t>prop-ex-m1-bike-bubble-r2.webp</t>
         </is>
       </c>
       <c r="G81" s="2" t="n"/>
@@ -4074,7 +4073,7 @@
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
-          <t>prop-ex-m1-wallet-r1.webp</t>
+          <t>prop-ex-m1-wallet-r2.webp</t>
         </is>
       </c>
       <c r="G88" s="2" t="inlineStr">
@@ -4409,7 +4408,7 @@
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
-          <t>prop-ex-m1-bike-bubble-r1.webp</t>
+          <t>prop-ex-m1-bike-bubble-r2.webp</t>
         </is>
       </c>
       <c r="G96" s="2" t="inlineStr">
@@ -4619,7 +4618,7 @@
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
-          <t>prop-ex-m1-wallet-r1.webp</t>
+          <t>prop-ex-m1-wallet-r2.webp</t>
         </is>
       </c>
       <c r="G101" s="2" t="inlineStr">
@@ -4960,7 +4959,7 @@
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
-          <t>prop-ex-m1-stand-set-r1.webp</t>
+          <t>prop-ex-m1-stand-set-r2.webp</t>
         </is>
       </c>
       <c r="G109" s="2" t="inlineStr">
@@ -5058,422 +5057,6 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A57"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
-  <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="16" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Explorer Image</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="16" customHeight="1">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>lemonade-family-scene-r10.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="32" customHeight="1">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>explorer-m1-l1-intro-lars-family-r2.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="16" customHeight="1">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>lars-senna-chatting.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="16" customHeight="1">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>concept-coin-stack.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="16" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>concept-wallet.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="16" customHeight="1">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>em1-02-l1r7-senna-coins-r3.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="16" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>concept-piggy-bank.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>lars-senna-sidebyside.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="32" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>em1-03-l1r11-lars-lemonade-r3.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="16" customHeight="1">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>medal-skill1-bronze-app.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="16" customHeight="1">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>beat-ex-m1-l2-r1.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="16" customHeight="1">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>concept-gift-box.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="32" customHeight="1">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>em1-05-l2r21-lars-mom-supplies-r1.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="16" customHeight="1">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>prop-ex-m1-wallet-r1.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="16" customHeight="1">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>lars-deciding-512.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="32" customHeight="1">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>em1-04-l2r20-lars-mom-bike-note-r3.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="16" customHeight="1">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>prop-ex-m1-stand-set-r1.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="16" customHeight="1">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>medal-skill2-bronze-app.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="16" customHeight="1">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>beat-ex-m1-l3-r1.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="32" customHeight="1">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>prop-ex-m1-emergencies-jar-r1.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="32" customHeight="1">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>em1-06-l3r27-emergencies-jar-r1.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="16" customHeight="1">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>lars-mason-chatting-512.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="24" ht="16" customHeight="1">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>medal-skill3-bronze.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="16" customHeight="1">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>beat-ex-m1-l4-r1.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="16" customHeight="1">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>lars-mason-sidebyside-512.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="16" customHeight="1">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>lars-mason-chatting.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="32" customHeight="1">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>em1-09-l4r41-saving-stand-dream-r1.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="16" customHeight="1">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>fishing-rod-sign.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="16" customHeight="1">
-      <c r="A30" s="2" t="inlineStr">
-        <is>
-          <t>concept-growth-chart.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="32" customHeight="1">
-      <c r="A31" s="2" t="inlineStr">
-        <is>
-          <t>em1-08-l4r45-startup-envelope-r3.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="16" customHeight="1">
-      <c r="A32" s="2" t="inlineStr">
-        <is>
-          <t>medal-skill1-silver.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="16" customHeight="1">
-      <c r="A33" s="2" t="inlineStr">
-        <is>
-          <t>beat-ex-m1-l5-r4.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="16" customHeight="1">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>lars-mia-sidebyside.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="32" customHeight="1">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>em1-10-l5r50-lars-mia-gelato-r1.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="16" customHeight="1">
-      <c r="A36" s="2" t="inlineStr">
-        <is>
-          <t>lars-thinking-512.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="16" customHeight="1">
-      <c r="A37" s="2" t="inlineStr">
-        <is>
-          <t>prop-ex-m1-gelato-r3.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="16" customHeight="1">
-      <c r="A38" s="2" t="inlineStr">
-        <is>
-          <t>lars-mia-chatting.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="16" customHeight="1">
-      <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t>medal-skill2-silver.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="16" customHeight="1">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>beat-ex-m1-l6-r1.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="32" customHeight="1">
-      <c r="A41" s="2" t="inlineStr">
-        <is>
-          <t>em1-11-l6r59-lars-movie-ticket-r1.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="32" customHeight="1">
-      <c r="A42" s="2" t="inlineStr">
-        <is>
-          <t>em1-12-l6r60-mia-lemon-doodle-r1.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="16" customHeight="1">
-      <c r="A43" s="2" t="inlineStr">
-        <is>
-          <t>prop-ex-m1-lemon-ticket-r4.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="16" customHeight="1">
-      <c r="A44" s="2" t="inlineStr">
-        <is>
-          <t>medal-skill3-silver.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="16" customHeight="1">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>beat-ex-m1-l7-r1.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="32" customHeight="1">
-      <c r="A46" s="2" t="inlineStr">
-        <is>
-          <t>em1-15-l7r72-lars-bike-dream-r1.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="32" customHeight="1">
-      <c r="A47" s="2" t="inlineStr">
-        <is>
-          <t>em1-16-l7r73-lars-wallet-mall-r1.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="16" customHeight="1">
-      <c r="A48" s="2" t="inlineStr">
-        <is>
-          <t>prop-ex-m1-slushie-r2.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="16" customHeight="1">
-      <c r="A49" s="2" t="inlineStr">
-        <is>
-          <t>lars-waving-512.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="16" customHeight="1">
-      <c r="A50" s="2" t="inlineStr">
-        <is>
-          <t>prop-ex-m1-bike-bubble-r1.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="16" customHeight="1">
-      <c r="A51" s="2" t="inlineStr">
-        <is>
-          <t>beat-ex-m1-l8-r2.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="16" customHeight="1">
-      <c r="A52" s="2" t="inlineStr">
-        <is>
-          <t>lars-mason-sidebyside.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="32" customHeight="1">
-      <c r="A53" s="2" t="inlineStr">
-        <is>
-          <t>em1-07-l3r31-lars-mason-empty-wallet-r1.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="32" customHeight="1">
-      <c r="A54" s="2" t="inlineStr">
-        <is>
-          <t>em1-18-l9r103-lars-closer-to-bike-r1.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="16" customHeight="1">
-      <c r="A55" s="2" t="inlineStr">
-        <is>
-          <t>beat-ex-m1-l9-r1.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="32" customHeight="1">
-      <c r="A56" s="2" t="inlineStr">
-        <is>
-          <t>em1-17-l9r102-lemonade-stand-open-r1.webp</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="16" customHeight="1">
-      <c r="A57" s="2" t="inlineStr">
-        <is>
-          <t>lars-celebrating-512.webp</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6151,7 +5734,7 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>prop-pf-m1-startup-kit-r2.webp</t>
+          <t>prop-pf-m1-startup-kit-r3.webp</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
@@ -6195,7 +5778,7 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>prop-ex-m1-wallet-r1.webp</t>
+          <t>prop-ex-m1-wallet-r2.webp</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">
@@ -6439,7 +6022,7 @@
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>prop-pf-m1-startup-kit-r2.webp</t>
+          <t>prop-pf-m1-startup-kit-r3.webp</t>
         </is>
       </c>
       <c r="G23" s="5" t="n"/>
@@ -6721,7 +6304,7 @@
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>prop-ex-m1-emergencies-jar-r1.webp</t>
+          <t>prop-ex-m1-emergencies-jar-r2.webp</t>
         </is>
       </c>
       <c r="G30" s="5" t="n"/>
@@ -7127,7 +6710,7 @@
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>prop-pf-m1-startup-kit-r2.webp</t>
+          <t>prop-pf-m1-startup-kit-r3.webp</t>
         </is>
       </c>
       <c r="G40" s="5" t="n"/>
@@ -7382,7 +6965,7 @@
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>prop-pf-m1-startup-kit-r2.webp</t>
+          <t>prop-pf-m1-startup-kit-r3.webp</t>
         </is>
       </c>
       <c r="G46" s="5" t="n"/>
@@ -7628,7 +7211,7 @@
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>prop-ex-m1-gelato-r3.webp</t>
+          <t>prop-ex-m1-gelato-r4.webp</t>
         </is>
       </c>
       <c r="G52" s="5" t="inlineStr">
@@ -7707,7 +7290,7 @@
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>prop-ex-m1-wallet-r1.webp</t>
+          <t>prop-ex-m1-wallet-r2.webp</t>
         </is>
       </c>
       <c r="G54" s="5" t="inlineStr">
@@ -7985,7 +7568,7 @@
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>prop-pf-m1-paw-ticket-r2.webp</t>
+          <t>prop-pf-m1-paw-ticket-r3.webp</t>
         </is>
       </c>
       <c r="G61" s="5" t="inlineStr">
@@ -8202,7 +7785,7 @@
       </c>
       <c r="F66" s="5" t="inlineStr">
         <is>
-          <t>prop-pf-m1-paw-ticket-r2.webp</t>
+          <t>prop-pf-m1-paw-ticket-r3.webp</t>
         </is>
       </c>
       <c r="G66" s="5" t="n"/>
@@ -8313,7 +7896,7 @@
       </c>
       <c r="F69" s="5" t="inlineStr">
         <is>
-          <t>prop-pf-m1-paw-ticket-r2.webp</t>
+          <t>prop-pf-m1-paw-ticket-r3.webp</t>
         </is>
       </c>
       <c r="G69" s="5" t="n"/>
@@ -8467,7 +8050,7 @@
       </c>
       <c r="F73" s="5" t="inlineStr">
         <is>
-          <t>prop-pf-m1-trip-bubble-r1.webp</t>
+          <t>prop-pf-m1-trip-bubble-r2.webp</t>
         </is>
       </c>
       <c r="G73" s="5" t="inlineStr">
@@ -8510,7 +8093,7 @@
       </c>
       <c r="F74" s="5" t="inlineStr">
         <is>
-          <t>prop-ex-m1-wallet-r1.webp</t>
+          <t>prop-ex-m1-wallet-r2.webp</t>
         </is>
       </c>
       <c r="G74" s="5" t="inlineStr">
@@ -8722,7 +8305,7 @@
       </c>
       <c r="F79" s="5" t="inlineStr">
         <is>
-          <t>prop-pf-m1-bubble-tea-r1.webp</t>
+          <t>prop-pf-m1-bubble-tea-r2.webp</t>
         </is>
       </c>
       <c r="G79" s="5" t="n"/>
@@ -8793,7 +8376,7 @@
       </c>
       <c r="F81" s="5" t="inlineStr">
         <is>
-          <t>prop-pf-m1-trip-bubble-r1.webp</t>
+          <t>prop-pf-m1-trip-bubble-r2.webp</t>
         </is>
       </c>
       <c r="G81" s="5" t="n"/>
@@ -8910,7 +8493,7 @@
       </c>
       <c r="F84" s="5" t="inlineStr">
         <is>
-          <t>prop-ex-m1-wallet-r1.webp</t>
+          <t>prop-ex-m1-wallet-r2.webp</t>
         </is>
       </c>
       <c r="G84" s="5" t="inlineStr">
@@ -9080,7 +8663,7 @@
       </c>
       <c r="F88" s="5" t="inlineStr">
         <is>
-          <t>prop-ex-m1-wallet-r1.webp</t>
+          <t>prop-ex-m1-wallet-r2.webp</t>
         </is>
       </c>
       <c r="G88" s="5" t="inlineStr">
@@ -9411,7 +8994,7 @@
       </c>
       <c r="F96" s="5" t="inlineStr">
         <is>
-          <t>prop-pf-m1-trip-bubble-r1.webp</t>
+          <t>prop-pf-m1-trip-bubble-r2.webp</t>
         </is>
       </c>
       <c r="G96" s="5" t="inlineStr">
@@ -9621,7 +9204,7 @@
       </c>
       <c r="F101" s="5" t="inlineStr">
         <is>
-          <t>prop-ex-m1-wallet-r1.webp</t>
+          <t>prop-ex-m1-wallet-r2.webp</t>
         </is>
       </c>
       <c r="G101" s="5" t="inlineStr">
@@ -9699,7 +9282,7 @@
       </c>
       <c r="F103" s="5" t="inlineStr">
         <is>
-          <t>prop-pf-m1-trip-bubble-r1.webp</t>
+          <t>prop-pf-m1-trip-bubble-r2.webp</t>
         </is>
       </c>
       <c r="G103" s="5" t="inlineStr">
@@ -9915,7 +9498,7 @@
       </c>
       <c r="F108" s="5" t="inlineStr">
         <is>
-          <t>prop-pf-m1-beagle-r1.webp</t>
+          <t>prop-pf-m1-beagle-r2.webp</t>
         </is>
       </c>
       <c r="G108" s="5" t="inlineStr">
@@ -9962,7 +9545,7 @@
       </c>
       <c r="F109" s="5" t="inlineStr">
         <is>
-          <t>prop-pf-m1-startup-kit-r2.webp</t>
+          <t>prop-pf-m1-startup-kit-r3.webp</t>
         </is>
       </c>
       <c r="G109" s="5" t="inlineStr">
@@ -10059,7 +9642,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -10079,8 +9662,8 @@
     <col width="50" customWidth="1" style="6" min="9" max="9"/>
     <col width="45" customWidth="1" style="6" min="10" max="10"/>
     <col width="18" customWidth="1" style="6" min="11" max="11"/>
-    <col width="8.83203125" customWidth="1" style="6" min="12" max="15"/>
-    <col width="8.83203125" customWidth="1" style="6" min="16" max="16384"/>
+    <col width="8.83203125" customWidth="1" style="6" min="12" max="16"/>
+    <col width="8.83203125" customWidth="1" style="6" min="17" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -10351,7 +9934,7 @@
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>prop-mv-m1-group-money-r1-app.webp</t>
+          <t>prop-mv-m1-group-money-r2-app.webp</t>
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr">
@@ -10506,7 +10089,7 @@
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>prop-mv-m1-tripod-r1-app.webp</t>
+          <t>prop-mv-m1-tripod-r2-app.webp</t>
         </is>
       </c>
       <c r="I11" s="6" t="inlineStr">
@@ -10691,7 +10274,7 @@
       </c>
       <c r="F16" s="6" t="inlineStr">
         <is>
-          <t>prop-mv-m1-tripod-r1-app.webp</t>
+          <t>prop-mv-m1-tripod-r2-app.webp</t>
         </is>
       </c>
       <c r="G16" s="6" t="inlineStr">
@@ -10731,7 +10314,7 @@
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
-          <t>prop-ex-m1-wallet-r1.webp</t>
+          <t>prop-ex-m1-wallet-r2.webp</t>
         </is>
       </c>
       <c r="G17" s="6" t="inlineStr">
@@ -10919,7 +10502,7 @@
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>prop-mv-m1-group-plan-r1-app.webp</t>
+          <t>prop-mv-m1-group-plan-r2-app.webp</t>
         </is>
       </c>
       <c r="I22" s="6" t="inlineStr">
@@ -10952,7 +10535,7 @@
       </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
-          <t>prop-mv-m1-group-startup-kit-r2-app.webp</t>
+          <t>prop-mv-m1-group-startup-kit-r3-app.webp</t>
         </is>
       </c>
       <c r="K23" s="6" t="inlineStr">
@@ -11201,7 +10784,7 @@
       </c>
       <c r="F30" s="6" t="inlineStr">
         <is>
-          <t>prop-ex-m1-wallet-r1.webp</t>
+          <t>prop-ex-m1-wallet-r2.webp</t>
         </is>
       </c>
       <c r="K30" s="6" t="inlineStr">
@@ -11283,7 +10866,7 @@
       </c>
       <c r="F32" s="6" t="inlineStr">
         <is>
-          <t>prop-mv-m1-group-headphones-r1-app.webp</t>
+          <t>prop-mv-m1-group-headphones-r2-app.webp</t>
         </is>
       </c>
       <c r="G32" s="6" t="inlineStr">
@@ -11566,7 +11149,7 @@
       </c>
       <c r="F40" s="6" t="inlineStr">
         <is>
-          <t>prop-mv-m1-group-startup-kit-r2-app.webp</t>
+          <t>prop-mv-m1-group-startup-kit-r3-app.webp</t>
         </is>
       </c>
       <c r="K40" s="6" t="inlineStr">
@@ -11767,7 +11350,7 @@
       </c>
       <c r="F45" s="6" t="inlineStr">
         <is>
-          <t>prop-mv-m1-group-money-r1-app.webp</t>
+          <t>prop-mv-m1-group-money-r2-app.webp</t>
         </is>
       </c>
       <c r="K45" s="6" t="inlineStr">
@@ -11795,7 +11378,7 @@
       </c>
       <c r="F46" s="6" t="inlineStr">
         <is>
-          <t>prop-mv-m1-group-startup-kit-r2-app.webp</t>
+          <t>prop-mv-m1-group-startup-kit-r3-app.webp</t>
         </is>
       </c>
       <c r="K46" s="6" t="inlineStr">
@@ -11935,7 +11518,7 @@
       </c>
       <c r="F50" s="6" t="inlineStr">
         <is>
-          <t>prop-mv-m1-group-startup-kit-r2-app.webp</t>
+          <t>prop-mv-m1-group-startup-kit-r3-app.webp</t>
         </is>
       </c>
       <c r="G50" s="6" t="inlineStr">
@@ -12016,7 +11599,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>prop-ex-m1-gelato-r3.webp</t>
+          <t>prop-ex-m1-gelato-r4.webp</t>
         </is>
       </c>
       <c r="G52" s="6" t="inlineStr">
@@ -12085,7 +11668,7 @@
       </c>
       <c r="F54" s="6" t="inlineStr">
         <is>
-          <t>prop-ex-m1-wallet-r1.webp</t>
+          <t>prop-ex-m1-wallet-r2.webp</t>
         </is>
       </c>
       <c r="G54" s="6" t="inlineStr">
@@ -12335,7 +11918,7 @@
       </c>
       <c r="F61" s="6" t="inlineStr">
         <is>
-          <t>prop-mv-m1-camera-ticket-r2.webp</t>
+          <t>prop-mv-m1-camera-ticket-r3.webp</t>
         </is>
       </c>
       <c r="G61" s="6" t="inlineStr">
@@ -12456,7 +12039,7 @@
       </c>
       <c r="F64" s="6" t="inlineStr">
         <is>
-          <t>prop-mv-m1-group-movie-day-r2-app.webp</t>
+          <t>prop-mv-m1-group-movie-day-r3-app.webp</t>
         </is>
       </c>
       <c r="G64" s="6" t="inlineStr">
@@ -12531,7 +12114,7 @@
       </c>
       <c r="F66" s="6" t="inlineStr">
         <is>
-          <t>prop-mv-m1-camera-ticket-r2.webp</t>
+          <t>prop-mv-m1-camera-ticket-r3.webp</t>
         </is>
       </c>
       <c r="K66" s="6" t="inlineStr">
@@ -12626,7 +12209,7 @@
       </c>
       <c r="F69" s="6" t="inlineStr">
         <is>
-          <t>prop-mv-m1-camera-ticket-r2.webp</t>
+          <t>prop-mv-m1-camera-ticket-r3.webp</t>
         </is>
       </c>
       <c r="K69" s="6" t="inlineStr">
@@ -12761,7 +12344,7 @@
       </c>
       <c r="F73" s="6" t="inlineStr">
         <is>
-          <t>prop-mv-m1-camera-bubble-r2.webp</t>
+          <t>prop-mv-m1-camera-bubble-r3.webp</t>
         </is>
       </c>
       <c r="G73" s="6" t="inlineStr">
@@ -12800,7 +12383,7 @@
       </c>
       <c r="F74" s="6" t="inlineStr">
         <is>
-          <t>prop-mv-m1-group-money-r1-app.webp</t>
+          <t>prop-mv-m1-group-money-r2-app.webp</t>
         </is>
       </c>
       <c r="G74" s="6" t="inlineStr">
@@ -12991,7 +12574,7 @@
       </c>
       <c r="F79" s="6" t="inlineStr">
         <is>
-          <t>prop-mv-m1-smoothie-r1.webp</t>
+          <t>prop-mv-m1-smoothie-r2.webp</t>
         </is>
       </c>
       <c r="K79" s="6" t="inlineStr">
@@ -13051,7 +12634,7 @@
       </c>
       <c r="F81" s="6" t="inlineStr">
         <is>
-          <t>prop-mv-m1-camera-bubble-r2.webp</t>
+          <t>prop-mv-m1-camera-bubble-r3.webp</t>
         </is>
       </c>
       <c r="K81" s="6" t="inlineStr">
@@ -13154,7 +12737,7 @@
       </c>
       <c r="F84" s="6" t="inlineStr">
         <is>
-          <t>prop-mv-m1-group-money-r1-app.webp</t>
+          <t>prop-mv-m1-group-money-r2-app.webp</t>
         </is>
       </c>
       <c r="G84" s="6" t="inlineStr">
@@ -13308,7 +12891,7 @@
       </c>
       <c r="F88" s="6" t="inlineStr">
         <is>
-          <t>prop-ex-m1-wallet-r1.webp</t>
+          <t>prop-ex-m1-wallet-r2.webp</t>
         </is>
       </c>
       <c r="G88" s="6" t="inlineStr">
@@ -13612,7 +13195,7 @@
       </c>
       <c r="F96" s="6" t="inlineStr">
         <is>
-          <t>prop-mv-m1-camera-bubble-r2.webp</t>
+          <t>prop-mv-m1-camera-bubble-r3.webp</t>
         </is>
       </c>
       <c r="G96" s="6" t="inlineStr">
@@ -13802,7 +13385,7 @@
       </c>
       <c r="F101" s="6" t="inlineStr">
         <is>
-          <t>prop-ex-m1-wallet-r1.webp</t>
+          <t>prop-ex-m1-wallet-r2.webp</t>
         </is>
       </c>
       <c r="G101" s="6" t="inlineStr">
@@ -13871,7 +13454,7 @@
       </c>
       <c r="F103" s="6" t="inlineStr">
         <is>
-          <t>prop-mv-m1-camera-bubble-r2.webp</t>
+          <t>prop-mv-m1-camera-bubble-r3.webp</t>
         </is>
       </c>
       <c r="G103" s="6" t="inlineStr">
@@ -14067,7 +13650,7 @@
       </c>
       <c r="F108" s="6" t="inlineStr">
         <is>
-          <t>prop-mv-m1-tripod-r1-app.webp</t>
+          <t>prop-mv-m1-tripod-r2-app.webp</t>
         </is>
       </c>
       <c r="G108" s="6" t="inlineStr">
@@ -14111,7 +13694,7 @@
       </c>
       <c r="F109" s="6" t="inlineStr">
         <is>
-          <t>prop-mv-m1-group-startup-kit-r2-app.webp</t>
+          <t>prop-mv-m1-group-startup-kit-r3-app.webp</t>
         </is>
       </c>
       <c r="G109" s="6" t="inlineStr">
@@ -14194,7 +13777,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -14214,8 +13797,8 @@
     <col width="50" customWidth="1" style="6" min="9" max="9"/>
     <col width="45" customWidth="1" style="6" min="10" max="10"/>
     <col width="18" customWidth="1" style="6" min="11" max="11"/>
-    <col width="8.83203125" customWidth="1" style="6" min="12" max="12"/>
-    <col width="8.83203125" customWidth="1" style="6" min="13" max="16384"/>
+    <col width="8.83203125" customWidth="1" style="6" min="12" max="13"/>
+    <col width="8.83203125" customWidth="1" style="6" min="14" max="16384"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -17538,7 +17121,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -20880,7 +20463,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -20965,7 +20548,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Bundle the Aiden name fix, round-2 props, and gold medals.
Preview reads master 225c3462. Maverick copy says Aiden, three Ara clips replace the retired takes, and column F names the round-2 props plus the new Aiden pair and beat art. Skills 1–3 gold medals use the round-2 files. The gift drag still targets max-celebrating.

Co-authored-by: ngaadmin <ngaadmin@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/lib/academy/lessons/payload/source/master/module-1-screens.xlsx
+++ b/lib/academy/lessons/payload/source/master/module-1-screens.xlsx
@@ -57,7 +57,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -67,6 +67,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
       </patternFill>
     </fill>
   </fills>
@@ -83,7 +89,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -105,6 +111,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -696,7 +705,7 @@
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>concept-coin-stack.webp</t>
+          <t>concept-coin-stack-r2.webp</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -741,7 +750,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>concept-wallet.webp</t>
+          <t>concept-wallet-r2.webp</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -867,7 +876,7 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>concept-piggy-bank.webp</t>
+          <t>concept-piggy-bank-r2.webp</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -983,7 +992,7 @@
       <c r="E12" s="2" t="n"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>medal-skill1-bronze-app.webp</t>
+          <t>medal-skill1-bronze-r2-app.webp</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
@@ -1099,7 +1108,7 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>concept-gift-box.webp</t>
+          <t>concept-gift-box-r2.webp</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -1267,7 +1276,7 @@
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>concept-piggy-bank.webp</t>
+          <t>concept-piggy-bank-r2.webp</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
@@ -1465,7 +1474,7 @@
       <c r="E24" s="2" t="n"/>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>medal-skill2-bronze-app.webp</t>
+          <t>medal-skill2-bronze-r2-app.webp</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -1584,7 +1593,7 @@
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>concept-wallet.webp</t>
+          <t>concept-wallet-r2.webp</t>
         </is>
       </c>
       <c r="G27" s="3" t="inlineStr">
@@ -1673,7 +1682,7 @@
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>concept-piggy-bank.webp</t>
+          <t>concept-piggy-bank-r2.webp</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -1916,7 +1925,7 @@
       <c r="E35" s="2" t="n"/>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>medal-skill3-bronze.webp</t>
+          <t>medal-skill3-bronze-r2.webp</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
@@ -2256,7 +2265,7 @@
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>concept-piggy-bank.webp</t>
+          <t>concept-piggy-bank-r2.webp</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
@@ -2301,7 +2310,7 @@
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
-          <t>concept-growth-chart.webp</t>
+          <t>concept-growth-chart-r2.webp</t>
         </is>
       </c>
       <c r="G44" s="2" t="inlineStr">
@@ -2408,7 +2417,7 @@
       <c r="E47" s="2" t="n"/>
       <c r="F47" s="2" t="inlineStr">
         <is>
-          <t>medal-skill1-silver.webp</t>
+          <t>medal-skill1-silver-r2.webp</t>
         </is>
       </c>
       <c r="G47" s="2" t="inlineStr">
@@ -2783,7 +2792,7 @@
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
-          <t>concept-piggy-bank.webp</t>
+          <t>concept-piggy-bank-r2.webp</t>
         </is>
       </c>
       <c r="G56" s="2" t="inlineStr">
@@ -2856,7 +2865,7 @@
       <c r="E58" s="2" t="n"/>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>medal-skill2-silver.webp</t>
+          <t>medal-skill2-silver-r2.webp</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -3018,7 +3027,7 @@
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t>concept-coin-stack.webp</t>
+          <t>concept-coin-stack-r2.webp</t>
         </is>
       </c>
       <c r="G62" s="4" t="inlineStr">
@@ -3155,7 +3164,7 @@
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
-          <t>concept-piggy-bank.webp</t>
+          <t>concept-piggy-bank-r2.webp</t>
         </is>
       </c>
       <c r="G65" s="2" t="inlineStr">
@@ -3339,7 +3348,7 @@
       <c r="E70" s="2" t="n"/>
       <c r="F70" s="2" t="inlineStr">
         <is>
-          <t>medal-skill3-silver.webp</t>
+          <t>medal-skill3-silver-r2.webp</t>
         </is>
       </c>
       <c r="G70" s="2" t="inlineStr">
@@ -3543,7 +3552,7 @@
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
-          <t>concept-coin-stack.webp</t>
+          <t>concept-coin-stack-r2.webp</t>
         </is>
       </c>
       <c r="G75" s="2" t="inlineStr">
@@ -3590,7 +3599,7 @@
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
-          <t>concept-wallet.webp</t>
+          <t>concept-wallet-r2.webp</t>
         </is>
       </c>
       <c r="G76" s="2" t="inlineStr">
@@ -3861,7 +3870,7 @@
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>concept-coin-stack.webp</t>
+          <t>concept-coin-stack-r2.webp</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
@@ -3944,7 +3953,7 @@
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
-          <t>concept-piggy-bank.webp</t>
+          <t>concept-piggy-bank-r2.webp</t>
         </is>
       </c>
       <c r="G85" s="2" t="inlineStr">
@@ -4114,7 +4123,7 @@
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
-          <t>concept-wallet.webp</t>
+          <t>concept-wallet-r2.webp</t>
         </is>
       </c>
       <c r="G89" s="2" t="inlineStr">
@@ -4283,7 +4292,7 @@
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
-          <t>concept-piggy-bank.webp</t>
+          <t>concept-piggy-bank-r2.webp</t>
         </is>
       </c>
       <c r="G93" s="2" t="inlineStr">
@@ -4324,7 +4333,7 @@
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
-          <t>concept-growth-chart.webp</t>
+          <t>concept-growth-chart-r2.webp</t>
         </is>
       </c>
       <c r="G94" s="2" t="inlineStr">
@@ -4495,7 +4504,7 @@
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
-          <t>concept-coin-stack.webp</t>
+          <t>concept-coin-stack-r2.webp</t>
         </is>
       </c>
       <c r="G98" s="2" t="inlineStr">
@@ -4536,7 +4545,7 @@
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
-          <t>concept-piggy-bank.webp</t>
+          <t>concept-piggy-bank-r2.webp</t>
         </is>
       </c>
       <c r="G99" s="2" t="inlineStr">
@@ -4784,7 +4793,7 @@
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
-          <t>concept-coin-stack.webp</t>
+          <t>concept-coin-stack-r2.webp</t>
         </is>
       </c>
       <c r="G105" s="2" t="inlineStr">
@@ -5286,7 +5295,7 @@
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>concept-coin-stack.webp</t>
+          <t>concept-coin-stack-r2.webp</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
@@ -5331,7 +5340,7 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>concept-wallet.webp</t>
+          <t>concept-wallet-r2.webp</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
@@ -5457,7 +5466,7 @@
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>concept-piggy-bank.webp</t>
+          <t>concept-piggy-bank-r2.webp</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
@@ -5573,7 +5582,7 @@
       <c r="E12" s="5" t="n"/>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>medal-skill1-bronze-app.webp</t>
+          <t>medal-skill1-bronze-r2-app.webp</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
@@ -5689,7 +5698,7 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>concept-gift-box.webp</t>
+          <t>concept-gift-box-r2.webp</t>
         </is>
       </c>
       <c r="G15" s="4" t="inlineStr">
@@ -5857,7 +5866,7 @@
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>concept-piggy-bank.webp</t>
+          <t>concept-piggy-bank-r2.webp</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
@@ -6059,7 +6068,7 @@
       <c r="E24" s="5" t="n"/>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>medal-skill2-bronze-app.webp</t>
+          <t>medal-skill2-bronze-r2-app.webp</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
@@ -6178,7 +6187,7 @@
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>concept-wallet.webp</t>
+          <t>concept-wallet-r2.webp</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
@@ -6267,7 +6276,7 @@
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>concept-piggy-bank.webp</t>
+          <t>concept-piggy-bank-r2.webp</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
@@ -6393,7 +6402,7 @@
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>concept-coin-stack.webp</t>
+          <t>concept-coin-stack-r2.webp</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
@@ -6510,7 +6519,7 @@
       <c r="E35" s="5" t="n"/>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>medal-skill3-bronze.webp</t>
+          <t>medal-skill3-bronze-r2.webp</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
@@ -6850,7 +6859,7 @@
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>concept-piggy-bank.webp</t>
+          <t>concept-piggy-bank-r2.webp</t>
         </is>
       </c>
       <c r="G43" s="5" t="inlineStr">
@@ -6895,7 +6904,7 @@
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>concept-growth-chart.webp</t>
+          <t>concept-growth-chart-r2.webp</t>
         </is>
       </c>
       <c r="G44" s="5" t="inlineStr">
@@ -7002,7 +7011,7 @@
       <c r="E47" s="5" t="n"/>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>medal-skill1-silver.webp</t>
+          <t>medal-skill1-silver-r2.webp</t>
         </is>
       </c>
       <c r="G47" s="5" t="inlineStr">
@@ -7377,7 +7386,7 @@
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>concept-piggy-bank.webp</t>
+          <t>concept-piggy-bank-r2.webp</t>
         </is>
       </c>
       <c r="G56" s="5" t="inlineStr">
@@ -7450,7 +7459,7 @@
       <c r="E58" s="5" t="n"/>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>medal-skill2-silver.webp</t>
+          <t>medal-skill2-silver-r2.webp</t>
         </is>
       </c>
       <c r="G58" s="5" t="inlineStr">
@@ -7612,7 +7621,7 @@
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>concept-coin-stack.webp</t>
+          <t>concept-coin-stack-r2.webp</t>
         </is>
       </c>
       <c r="G62" s="5" t="inlineStr">
@@ -7749,7 +7758,7 @@
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>concept-piggy-bank.webp</t>
+          <t>concept-piggy-bank-r2.webp</t>
         </is>
       </c>
       <c r="G65" s="5" t="inlineStr">
@@ -7933,7 +7942,7 @@
       <c r="E70" s="5" t="n"/>
       <c r="F70" s="5" t="inlineStr">
         <is>
-          <t>medal-skill3-silver.webp</t>
+          <t>medal-skill3-silver-r2.webp</t>
         </is>
       </c>
       <c r="G70" s="5" t="inlineStr">
@@ -8137,7 +8146,7 @@
       </c>
       <c r="F75" s="5" t="inlineStr">
         <is>
-          <t>concept-coin-stack.webp</t>
+          <t>concept-coin-stack-r2.webp</t>
         </is>
       </c>
       <c r="G75" s="5" t="inlineStr">
@@ -8184,7 +8193,7 @@
       </c>
       <c r="F76" s="5" t="inlineStr">
         <is>
-          <t>concept-wallet.webp</t>
+          <t>concept-wallet-r2.webp</t>
         </is>
       </c>
       <c r="G76" s="5" t="inlineStr">
@@ -8451,7 +8460,7 @@
       </c>
       <c r="F83" s="5" t="inlineStr">
         <is>
-          <t>concept-coin-stack.webp</t>
+          <t>concept-coin-stack-r2.webp</t>
         </is>
       </c>
       <c r="G83" s="5" t="inlineStr">
@@ -8534,7 +8543,7 @@
       </c>
       <c r="F85" s="5" t="inlineStr">
         <is>
-          <t>concept-piggy-bank.webp</t>
+          <t>concept-piggy-bank-r2.webp</t>
         </is>
       </c>
       <c r="G85" s="5" t="inlineStr">
@@ -8704,7 +8713,7 @@
       </c>
       <c r="F89" s="5" t="inlineStr">
         <is>
-          <t>concept-wallet.webp</t>
+          <t>concept-wallet-r2.webp</t>
         </is>
       </c>
       <c r="G89" s="5" t="inlineStr">
@@ -8869,7 +8878,7 @@
       </c>
       <c r="F93" s="5" t="inlineStr">
         <is>
-          <t>concept-piggy-bank.webp</t>
+          <t>concept-piggy-bank-r2.webp</t>
         </is>
       </c>
       <c r="G93" s="5" t="inlineStr">
@@ -8910,7 +8919,7 @@
       </c>
       <c r="F94" s="5" t="inlineStr">
         <is>
-          <t>concept-growth-chart.webp</t>
+          <t>concept-growth-chart-r2.webp</t>
         </is>
       </c>
       <c r="G94" s="5" t="inlineStr">
@@ -8953,7 +8962,7 @@
       </c>
       <c r="F95" s="5" t="inlineStr">
         <is>
-          <t>concept-wallet.webp</t>
+          <t>concept-wallet-r2.webp</t>
         </is>
       </c>
       <c r="G95" s="5" t="inlineStr">
@@ -9081,7 +9090,7 @@
       </c>
       <c r="F98" s="5" t="inlineStr">
         <is>
-          <t>concept-coin-stack.webp</t>
+          <t>concept-coin-stack-r2.webp</t>
         </is>
       </c>
       <c r="G98" s="5" t="inlineStr">
@@ -9122,7 +9131,7 @@
       </c>
       <c r="F99" s="5" t="inlineStr">
         <is>
-          <t>concept-piggy-bank.webp</t>
+          <t>concept-piggy-bank-r2.webp</t>
         </is>
       </c>
       <c r="G99" s="5" t="inlineStr">
@@ -9370,7 +9379,7 @@
       </c>
       <c r="F105" s="5" t="inlineStr">
         <is>
-          <t>concept-coin-stack.webp</t>
+          <t>concept-coin-stack-r2.webp</t>
         </is>
       </c>
       <c r="G105" s="5" t="inlineStr">
@@ -9861,7 +9870,7 @@
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>concept-coin-stack.webp</t>
+          <t>concept-coin-stack-r2.webp</t>
         </is>
       </c>
       <c r="G5" s="6" t="inlineStr">
@@ -9902,7 +9911,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>concept-wallet.webp</t>
+          <t>concept-wallet-r2.webp</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -10020,7 +10029,7 @@
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>concept-piggy-bank.webp</t>
+          <t>concept-piggy-bank-r2.webp</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr">
@@ -10126,7 +10135,7 @@
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>medal-skill1-bronze-app.webp</t>
+          <t>medal-skill1-bronze-r2-app.webp</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
@@ -10146,15 +10155,15 @@
           <t>Scenario Beat</t>
         </is>
       </c>
-      <c r="E13" s="6" t="inlineStr">
-        <is>
-          <t>Max's birthday is on Saturday, and Senna has a plan.
-He's going to get Max the power bank from the store window. There's just one problem...</t>
+      <c r="E13" s="8" t="inlineStr">
+        <is>
+          <t>Aiden's birthday is on Saturday, and Senna has a plan.
+He's going to get Aiden the power bank from the store window. There's just one problem...</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>beat-mv-m1-l2-r6-app.webp</t>
+          <t>beat-mv-m1-l2-r7-app.webp</t>
         </is>
       </c>
       <c r="I13" s="6" t="inlineStr">
@@ -10162,9 +10171,9 @@
           <t>Max fills Senna younger's (Explorer) L2/L3 role. Max: Senna older's friend, 17 per Cath 25 Oct.</t>
         </is>
       </c>
-      <c r="K13" s="6" t="inlineStr">
-        <is>
-          <t>maverick-m1-l1-beat3-f3e0e7b7.mp3</t>
+      <c r="K13" s="8" t="inlineStr">
+        <is>
+          <t>maverick-m1-l1-beat3-aa990a78.mp3</t>
         </is>
       </c>
     </row>
@@ -10189,14 +10198,14 @@
           <t>true-false</t>
         </is>
       </c>
-      <c r="E14" s="6" t="inlineStr">
-        <is>
-          <t>Senna promised Max a $30 power bank for his birthday on Saturday. Senna only has the $20 he kept safe. True or false: he can buy it now.</t>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>Senna promised Aiden a $30 power bank for his birthday on Saturday. Senna only has the $20 he kept safe. True or false: he can buy it now.</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>senna-older-max-chatting-r1-512.webp</t>
+          <t>senna-older-aiden19-chatting-r1-512.webp</t>
         </is>
       </c>
       <c r="G14" s="6" t="inlineStr">
@@ -10233,7 +10242,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>concept-gift-box.webp</t>
+          <t>concept-gift-box-r2.webp</t>
         </is>
       </c>
       <c r="G15" s="6" t="inlineStr">
@@ -10383,7 +10392,7 @@
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>concept-piggy-bank.webp</t>
+          <t>concept-piggy-bank-r2.webp</t>
         </is>
       </c>
       <c r="G19" s="6" t="inlineStr">
@@ -10460,21 +10469,21 @@
           <t>drag-to-target</t>
         </is>
       </c>
-      <c r="E21" s="6" t="inlineStr">
-        <is>
-          <t>It's Saturday, Max's birthday, and the party is about to start. Drag the gift to Max so Senna can keep his promise.</t>
+      <c r="E21" s="8" t="inlineStr">
+        <is>
+          <t>It's Saturday, Aiden's birthday, and the party is about to start. Drag the gift to Aiden so Senna can keep his promise.</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">
         <is>
-          <t>senna-older-max-sidebyside-r1-512.webp</t>
-        </is>
-      </c>
-      <c r="G21" s="6" t="inlineStr">
+          <t>senna-older-aiden19-sidebyside-r1-512.webp</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="inlineStr">
         <is>
           <t>SOURCE: concept-gift-box
 TARGET: max-celebrating
-SUCCESS: Promise kept! Happy birthday, Max! 🎉</t>
+SUCCESS: Promise kept! Happy birthday, Aiden! 🎉</t>
         </is>
       </c>
       <c r="I21" s="6" t="inlineStr">
@@ -10494,9 +10503,9 @@
           <t>Scenario Beat</t>
         </is>
       </c>
-      <c r="E22" s="6" t="inlineStr">
-        <is>
-          <t>Max loves his new power bank. That night, Senna tells Dad his big dream: a proper camera for filming content.
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>Aiden loves his new power bank. That night, Senna tells Dad his big dream: a proper camera for filming content.
 His parents say they'll help, but Senna has to pay for part of it himself. Spending money won't get him there, so Senna makes a plan.</t>
         </is>
       </c>
@@ -10510,9 +10519,9 @@
           <t>OPEN QUESTION: camera goal carried over from Cath's earlier Maverick draft; not set in the SoT.</t>
         </is>
       </c>
-      <c r="K22" s="6" t="inlineStr">
-        <is>
-          <t>maverick-m1-l2-beat2-1a2c4c12.mp3</t>
+      <c r="K22" s="8" t="inlineStr">
+        <is>
+          <t>maverick-m1-l2-beat2-c781b416.mp3</t>
         </is>
       </c>
     </row>
@@ -10567,7 +10576,7 @@
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>medal-skill2-bronze-app.webp</t>
+          <t>medal-skill2-bronze-r2-app.webp</t>
         </is>
       </c>
       <c r="G24" s="6" t="inlineStr">
@@ -10587,20 +10596,20 @@
           <t>Scenario Beat</t>
         </is>
       </c>
-      <c r="E25" s="6" t="inlineStr">
+      <c r="E25" s="8" t="inlineStr">
         <is>
           <t>Saving for his video kit sounds easy, but he keeps spending his money at the food court. The weeks fly by.
-Then one afternoon, Senna borrows Max's headphones...</t>
+Then one afternoon, Senna borrows Aiden's headphones...</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>beat-mv-m1-l3-r5-app.webp</t>
-        </is>
-      </c>
-      <c r="K25" s="6" t="inlineStr">
-        <is>
-          <t>maverick-m1-l2-beat4-e44a6ee7.mp3</t>
+          <t>beat-mv-m1-l3-r6-app.webp</t>
+        </is>
+      </c>
+      <c r="K25" s="8" t="inlineStr">
+        <is>
+          <t>maverick-m1-l2-beat4-c4dd707f.mp3</t>
         </is>
       </c>
     </row>
@@ -10625,14 +10634,14 @@
           <t>multiple-choice</t>
         </is>
       </c>
-      <c r="E26" s="6" t="inlineStr">
-        <is>
-          <t>He accidentally breaks Max's headphones. What's the problem Senna faces?</t>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>He accidentally breaks Aiden's headphones. What's the problem Senna faces?</t>
         </is>
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>senna-older-max-chatting-r1-512.webp</t>
+          <t>senna-older-aiden19-chatting-r1-512.webp</t>
         </is>
       </c>
       <c r="G26" s="6" t="inlineStr">
@@ -10672,7 +10681,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>concept-wallet.webp</t>
+          <t>concept-wallet-r2.webp</t>
         </is>
       </c>
       <c r="G27" s="6" t="inlineStr">
@@ -10706,14 +10715,14 @@
           <t>link-match</t>
         </is>
       </c>
-      <c r="E28" s="6" t="inlineStr">
-        <is>
-          <t>Max isn't upset for long, but Senna hates this feeling. Max says keeping Cash for Emergencies gives you choices. Match each event to what you could do.</t>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>Aiden isn't upset for long, but Senna hates this feeling. Aiden says keeping Cash for Emergencies gives you choices. Match each event to what you could do.</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>senna-older-max-sidebyside-r1-512.webp</t>
+          <t>senna-older-aiden19-sidebyside-r1-512.webp</t>
         </is>
       </c>
       <c r="G28" s="6" t="inlineStr">
@@ -10746,14 +10755,14 @@
           <t>rank-order</t>
         </is>
       </c>
-      <c r="E29" s="6" t="inlineStr">
-        <is>
-          <t>Max helps Senna make a plan, so he's never caught out again. Put the plan in order, first to last.</t>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>Aiden helps Senna make a plan, so he's never caught out again. Put the plan in order, first to last.</t>
         </is>
       </c>
       <c r="F29" s="6" t="inlineStr">
         <is>
-          <t>concept-piggy-bank.webp</t>
+          <t>concept-piggy-bank-r2.webp</t>
         </is>
       </c>
       <c r="G29" s="6" t="inlineStr">
@@ -10814,9 +10823,9 @@
           <t>multiple-choice</t>
         </is>
       </c>
-      <c r="E31" s="6" t="inlineStr">
-        <is>
-          <t>A few weeks later, Senna has saved $60, just enough for Max's new headphones. Then he sees a $20 wireless charger. "I'll buy it now and save more next week," he thinks. What should he do?</t>
+      <c r="E31" s="8" t="inlineStr">
+        <is>
+          <t>A few weeks later, Senna has saved $60, just enough for Aiden's new headphones. Then he sees a $20 wireless charger. "I'll buy it now and save more next week," he thinks. What should he do?</t>
         </is>
       </c>
       <c r="F31" s="6" t="inlineStr">
@@ -10824,10 +10833,10 @@
           <t>senna-older-deciding-r1-512.webp</t>
         </is>
       </c>
-      <c r="G31" s="6" t="inlineStr">
+      <c r="G31" s="8" t="inlineStr">
         <is>
           <t>CHOICE A: 🔌 Buy the charger and save $20 more next week.
-CHOICE B: 🎧 Buy Max's new headphones first.
+CHOICE B: 🎧 Buy Aiden's new headphones first.
 CHOICE C: 🤞 Buy the charger and hope headphones cost less.
 CORRECT: B</t>
         </is>
@@ -10859,9 +10868,9 @@
           <t>word-drop</t>
         </is>
       </c>
-      <c r="E32" s="6" t="inlineStr">
-        <is>
-          <t>Senna thinks: "Because I didn't ______ it all, I had cash to ______ Max's headphones right away."</t>
+      <c r="E32" s="8" t="inlineStr">
+        <is>
+          <t>Senna thinks: "Because I didn't ______ it all, I had cash to ______ Aiden's headphones right away."</t>
         </is>
       </c>
       <c r="F32" s="6" t="inlineStr">
@@ -10973,7 +10982,7 @@
       </c>
       <c r="F35" s="6" t="inlineStr">
         <is>
-          <t>medal-skill3-bronze.webp</t>
+          <t>medal-skill3-bronze-r2.webp</t>
         </is>
       </c>
       <c r="G35" s="6" t="inlineStr">
@@ -11279,7 +11288,7 @@
       </c>
       <c r="F43" s="6" t="inlineStr">
         <is>
-          <t>concept-piggy-bank.webp</t>
+          <t>concept-piggy-bank-r2.webp</t>
         </is>
       </c>
       <c r="G43" s="6" t="inlineStr">
@@ -11320,7 +11329,7 @@
       </c>
       <c r="F44" s="6" t="inlineStr">
         <is>
-          <t>concept-growth-chart.webp</t>
+          <t>concept-growth-chart-r2.webp</t>
         </is>
       </c>
       <c r="G44" s="6" t="inlineStr">
@@ -11410,7 +11419,7 @@
       </c>
       <c r="F47" s="6" t="inlineStr">
         <is>
-          <t>medal-skill1-silver.webp</t>
+          <t>medal-skill1-silver-r2.webp</t>
         </is>
       </c>
       <c r="G47" s="6" t="inlineStr">
@@ -11747,7 +11756,7 @@
       </c>
       <c r="F56" s="6" t="inlineStr">
         <is>
-          <t>concept-piggy-bank.webp</t>
+          <t>concept-piggy-bank-r2.webp</t>
         </is>
       </c>
       <c r="G56" s="6" t="inlineStr">
@@ -11809,7 +11818,7 @@
       </c>
       <c r="F58" s="6" t="inlineStr">
         <is>
-          <t>medal-skill2-silver.webp</t>
+          <t>medal-skill2-silver-r2.webp</t>
         </is>
       </c>
       <c r="G58" s="6" t="inlineStr">
@@ -11958,7 +11967,7 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>concept-coin-stack.webp</t>
+          <t>concept-coin-stack-r2.webp</t>
         </is>
       </c>
       <c r="G62" s="6" t="inlineStr">
@@ -12084,7 +12093,7 @@
       </c>
       <c r="F65" s="6" t="inlineStr">
         <is>
-          <t>concept-piggy-bank.webp</t>
+          <t>concept-piggy-bank-r2.webp</t>
         </is>
       </c>
       <c r="G65" s="6" t="inlineStr">
@@ -12241,7 +12250,7 @@
       </c>
       <c r="F70" s="6" t="inlineStr">
         <is>
-          <t>medal-skill3-silver.webp</t>
+          <t>medal-skill3-silver-r2.webp</t>
         </is>
       </c>
       <c r="G70" s="6" t="inlineStr">
@@ -12423,7 +12432,7 @@
       </c>
       <c r="F75" s="6" t="inlineStr">
         <is>
-          <t>concept-coin-stack.webp</t>
+          <t>concept-coin-stack-r2.webp</t>
         </is>
       </c>
       <c r="G75" s="6" t="inlineStr">
@@ -12467,7 +12476,7 @@
       </c>
       <c r="F76" s="6" t="inlineStr">
         <is>
-          <t>concept-wallet.webp</t>
+          <t>concept-wallet-r2.webp</t>
         </is>
       </c>
       <c r="G76" s="6" t="inlineStr">
@@ -12699,7 +12708,7 @@
       </c>
       <c r="F83" s="6" t="inlineStr">
         <is>
-          <t>concept-coin-stack.webp</t>
+          <t>concept-coin-stack-r2.webp</t>
         </is>
       </c>
       <c r="G83" s="6" t="inlineStr">
@@ -12774,7 +12783,7 @@
       </c>
       <c r="F85" s="6" t="inlineStr">
         <is>
-          <t>concept-piggy-bank.webp</t>
+          <t>concept-piggy-bank-r2.webp</t>
         </is>
       </c>
       <c r="G85" s="6" t="inlineStr">
@@ -12928,7 +12937,7 @@
       </c>
       <c r="F89" s="6" t="inlineStr">
         <is>
-          <t>concept-wallet.webp</t>
+          <t>concept-wallet-r2.webp</t>
         </is>
       </c>
       <c r="G89" s="6" t="inlineStr">
@@ -13082,7 +13091,7 @@
       </c>
       <c r="F93" s="6" t="inlineStr">
         <is>
-          <t>concept-piggy-bank.webp</t>
+          <t>concept-piggy-bank-r2.webp</t>
         </is>
       </c>
       <c r="G93" s="6" t="inlineStr">
@@ -13119,7 +13128,7 @@
       </c>
       <c r="F94" s="6" t="inlineStr">
         <is>
-          <t>concept-growth-chart.webp</t>
+          <t>concept-growth-chart-r2.webp</t>
         </is>
       </c>
       <c r="G94" s="6" t="inlineStr">
@@ -13158,7 +13167,7 @@
       </c>
       <c r="F95" s="6" t="inlineStr">
         <is>
-          <t>concept-wallet.webp</t>
+          <t>concept-wallet-r2.webp</t>
         </is>
       </c>
       <c r="G95" s="6" t="inlineStr">
@@ -13274,7 +13283,7 @@
       </c>
       <c r="F98" s="6" t="inlineStr">
         <is>
-          <t>concept-coin-stack.webp</t>
+          <t>concept-coin-stack-r2.webp</t>
         </is>
       </c>
       <c r="G98" s="6" t="inlineStr">
@@ -13311,7 +13320,7 @@
       </c>
       <c r="F99" s="6" t="inlineStr">
         <is>
-          <t>concept-piggy-bank.webp</t>
+          <t>concept-piggy-bank-r2.webp</t>
         </is>
       </c>
       <c r="G99" s="6" t="inlineStr">
@@ -13534,7 +13543,7 @@
       </c>
       <c r="F105" s="6" t="inlineStr">
         <is>
-          <t>concept-coin-stack.webp</t>
+          <t>concept-coin-stack-r2.webp</t>
         </is>
       </c>
       <c r="G105" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Relabel two lightning rows as binary choice.
Master d430777a changes column D on rows 8 and 54 in all three Module 1 tabs. Those settings already match the shared binary-choice mapping, so the column F picture shows.

Co-authored-by: ngaadmin <ngaadmin@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/lib/academy/lessons/payload/source/master/module-1-screens.xlsx
+++ b/lib/academy/lessons/payload/source/master/module-1-screens.xlsx
@@ -819,7 +819,7 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>spotlight-rounds</t>
+          <t>binary-choice</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
@@ -2695,7 +2695,7 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>spotlight-rounds</t>
+          <t>binary-choice</t>
         </is>
       </c>
       <c r="E54" s="4" t="inlineStr">
@@ -5409,7 +5409,7 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>spotlight-rounds</t>
+          <t>binary-choice</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -7289,7 +7289,7 @@
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>spotlight-rounds</t>
+          <t>binary-choice</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
@@ -9975,7 +9975,7 @@
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>spotlight-rounds</t>
+          <t>binary-choice</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
@@ -11667,7 +11667,7 @@
       </c>
       <c r="D54" s="6" t="inlineStr">
         <is>
-          <t>spotlight-rounds</t>
+          <t>binary-choice</t>
         </is>
       </c>
       <c r="E54" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Academy: Maverick M1 picture swaps off Max (10 cells, Jasper fix, Cath-approved, test only)
Master workbook md5 144a61a4d89043cadf45b0a0850cb55e. Only M1 Maverick column F
rows 49, 53, 55, 60, 67, 72, 77, 91, 92, 104 change; every name is already in
academy-media.
</commit_message>
<xml_diff>
--- a/lib/academy/lessons/payload/source/master/module-1-screens.xlsx
+++ b/lib/academy/lessons/payload/source/master/module-1-screens.xlsx
@@ -11615,7 +11615,7 @@
         <v>161</v>
       </c>
       <c r="F49" s="9" t="s">
-        <v>130</v>
+        <v>85</v>
       </c>
       <c r="G49" s="6" t="s">
         <v>162</v>
@@ -11704,7 +11704,7 @@
         <v>171</v>
       </c>
       <c r="F53" s="6" t="s">
-        <v>123</v>
+        <v>158</v>
       </c>
       <c r="K53" s="6" t="s">
         <v>172</v>
@@ -11750,7 +11750,7 @@
         <v>175</v>
       </c>
       <c r="F55" t="s">
-        <v>130</v>
+        <v>24</v>
       </c>
       <c r="G55" s="6" t="s">
         <v>176</v>
@@ -11850,7 +11850,7 @@
         <v>185</v>
       </c>
       <c r="F60" s="6" t="s">
-        <v>123</v>
+        <v>166</v>
       </c>
       <c r="G60" s="6" t="s">
         <v>186</v>
@@ -12011,7 +12011,7 @@
         <v>203</v>
       </c>
       <c r="F67" s="6" t="s">
-        <v>130</v>
+        <v>196</v>
       </c>
       <c r="G67" s="6" t="s">
         <v>204</v>
@@ -12105,7 +12105,7 @@
         <v>213</v>
       </c>
       <c r="F72" s="6" t="s">
-        <v>130</v>
+        <v>166</v>
       </c>
       <c r="G72" s="6" t="s">
         <v>214</v>
@@ -12223,7 +12223,7 @@
         <v>225</v>
       </c>
       <c r="F77" s="6" t="s">
-        <v>123</v>
+        <v>85</v>
       </c>
       <c r="G77" s="6" t="s">
         <v>226</v>
@@ -12524,7 +12524,7 @@
         <v>257</v>
       </c>
       <c r="F91" s="6" t="s">
-        <v>123</v>
+        <v>29</v>
       </c>
       <c r="G91" s="6" t="s">
         <v>258</v>
@@ -12550,7 +12550,7 @@
         <v>260</v>
       </c>
       <c r="F92" s="6" t="s">
-        <v>130</v>
+        <v>34</v>
       </c>
       <c r="G92" s="6" t="s">
         <v>261</v>
@@ -12823,7 +12823,7 @@
         <v>284</v>
       </c>
       <c r="F104" s="6" t="s">
-        <v>123</v>
+        <v>166</v>
       </c>
       <c r="G104" s="6" t="s">
         <v>285</v>

</xml_diff>